<commit_message>
removed facial recognition experiment and hardware update
</commit_message>
<xml_diff>
--- a/docs/Group6_PRG381_Project_RequiredHardware.xlsx
+++ b/docs/Group6_PRG381_Project_RequiredHardware.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerem\OneDrive\Desktop\cogniflight-edge\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F7F2B9C-BF6F-4DC5-BBE2-BDD76FAE4D9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C3ADEAC-5B9C-491B-B575-01142CDDA98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7BD184DE-096E-4408-BB28-F2172AC6A2E6}"/>
   </bookViews>
@@ -62,9 +62,6 @@
     <t>Execute ML inference (TensorFlow Lite), run OpenCV pipelines</t>
   </si>
   <si>
-    <t>Raspberry Pi 4 Model B (8 GB RAM)</t>
-  </si>
-  <si>
     <t>Cooling Fan</t>
   </si>
   <si>
@@ -89,9 +86,6 @@
     <t>Camera Module</t>
   </si>
   <si>
-    <t>Facial recognition, eye-blink &amp; yawning detection, night vision</t>
-  </si>
-  <si>
     <t>Storage &amp; Power</t>
   </si>
   <si>
@@ -107,12 +101,6 @@
     <t>Power Supply</t>
   </si>
   <si>
-    <t>Stable 5 V power for Pi 4 and peripherals</t>
-  </si>
-  <si>
-    <t>SMPS 5 V, 3 A (compatible with Raspberry Pi 4)</t>
-  </si>
-  <si>
     <t>Biosensors</t>
   </si>
   <si>
@@ -206,19 +194,31 @@
     <t>Assorted kit: 0.1 µF ceramic (X7R0104K52T),10 µF electrolytic (&gt;=10V)</t>
   </si>
   <si>
-    <t>Heatsink Kit</t>
-  </si>
-  <si>
-    <t>Raspberry Pi 4 Heatsink Set (3-pack)</t>
-  </si>
-  <si>
-    <t>Passive cooling for CPU</t>
-  </si>
-  <si>
-    <t>HKD FANDC005030-07</t>
-  </si>
-  <si>
     <t>RASPBERRY PI CAM MODULE 3W NOIR</t>
+  </si>
+  <si>
+    <t>5B camera cable</t>
+  </si>
+  <si>
+    <t>RASPBERRY PI 5B 16GB</t>
+  </si>
+  <si>
+    <t>RASPBERRY PI 5B active cooler</t>
+  </si>
+  <si>
+    <t>RASPBERRY PI 5B PSU 5V 5A TYPE-C</t>
+  </si>
+  <si>
+    <t>Stable 5 V power for Pi 5 and peripherals</t>
+  </si>
+  <si>
+    <t>camera cable</t>
+  </si>
+  <si>
+    <t>camera adapter cable</t>
+  </si>
+  <si>
+    <t>Facial recognition, eye-blink &amp; yawning detection</t>
   </si>
 </sst>
 </file>
@@ -641,7 +641,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -655,13 +655,13 @@
         <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="E2" s="3">
-        <v>2003.3</v>
+        <v>3180</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
@@ -669,19 +669,19 @@
         <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E3" s="3">
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -689,193 +689,193 @@
         <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="F4" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="C5" s="2" t="s">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E5" s="3">
         <v>816.5</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="E6" s="3">
         <v>75</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="E7" s="3">
-        <v>161</v>
+        <v>299</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E8" s="3">
         <v>990</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E9" s="3">
         <v>21</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E10" s="3">
         <v>10.01</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E11" s="3">
         <v>12</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="E12" s="4">
         <v>79.010000000000005</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E13" s="5">
         <v>20</v>
@@ -883,42 +883,42 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="E14" s="4">
         <v>12.28</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" t="s">
         <v>44</v>
       </c>
-      <c r="B15" t="s">
-        <v>48</v>
-      </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E15" s="5">
         <v>3</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -926,25 +926,25 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D16" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E16" s="5">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E17" s="4">
         <f>SUM(E2:E16)</f>
-        <v>4261.1000000000004</v>
+        <v>5662.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>